<commit_message>
feat: stabilize enterprise llm evaluation framework
</commit_message>
<xml_diff>
--- a/datasets/Login_test_repository.xlsx
+++ b/datasets/Login_test_repository.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shivani Rampally\DeepEval-POC\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DBCCD32B-32DB-4E88-8431-CBC94FAEFD87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A857EEB-6045-4440-8AA5-A6BBB47C4BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_Requirements" sheetId="1" r:id="rId1"/>
@@ -27,21 +27,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="235">
   <si>
-    <t>Requirement ID</t>
-  </si>
-  <si>
-    <t>Requirement Type</t>
-  </si>
-  <si>
     <t>Title</t>
   </si>
   <si>
-    <t>Description/Acceptance Criteria</t>
-  </si>
-  <si>
-    <t>Business Rules</t>
-  </si>
-  <si>
     <t>Priority</t>
   </si>
   <si>
@@ -730,6 +718,18 @@
   </si>
   <si>
     <t>Login response time</t>
+  </si>
+  <si>
+    <t>RequirementID</t>
+  </si>
+  <si>
+    <t>RequirementType</t>
+  </si>
+  <si>
+    <t>Description/AcceptanceCriteria</t>
+  </si>
+  <si>
+    <t>BusinessRules</t>
   </si>
 </sst>
 </file>
@@ -1094,144 +1094,144 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" t="s">
         <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
       <c r="D4" s="3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F4" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F7" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F8" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1258,642 +1258,642 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" t="s">
         <v>41</v>
       </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="H2" t="s">
         <v>42</v>
       </c>
-      <c r="D2" t="s">
+      <c r="I2" t="s">
         <v>43</v>
       </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="J2" t="s">
         <v>44</v>
-      </c>
-      <c r="G2" t="s">
-        <v>45</v>
-      </c>
-      <c r="H2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I2" t="s">
-        <v>47</v>
-      </c>
-      <c r="J2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3" t="s">
+        <v>41</v>
+      </c>
+      <c r="H3" t="s">
         <v>42</v>
       </c>
-      <c r="D3" t="s">
-        <v>43</v>
-      </c>
-      <c r="E3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" t="s">
-        <v>50</v>
-      </c>
-      <c r="G3" t="s">
-        <v>45</v>
-      </c>
-      <c r="H3" t="s">
-        <v>46</v>
-      </c>
       <c r="I3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="J3" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" t="s">
+        <v>50</v>
+      </c>
+      <c r="G4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H4" t="s">
         <v>42</v>
       </c>
-      <c r="D4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" t="s">
-        <v>54</v>
-      </c>
-      <c r="G4" t="s">
-        <v>45</v>
-      </c>
-      <c r="H4" t="s">
-        <v>46</v>
-      </c>
       <c r="I4" t="s">
+        <v>47</v>
+      </c>
+      <c r="J4" t="s">
         <v>51</v>
-      </c>
-      <c r="J4" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" t="s">
+        <v>55</v>
+      </c>
+      <c r="G5" t="s">
         <v>56</v>
       </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="H5" t="s">
         <v>57</v>
       </c>
-      <c r="D5" t="s">
+      <c r="I5" t="s">
         <v>58</v>
       </c>
-      <c r="E5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="J5" t="s">
         <v>59</v>
-      </c>
-      <c r="G5" t="s">
-        <v>60</v>
-      </c>
-      <c r="H5" t="s">
-        <v>61</v>
-      </c>
-      <c r="I5" t="s">
-        <v>62</v>
-      </c>
-      <c r="J5" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F6" t="s">
+        <v>61</v>
+      </c>
+      <c r="G6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H6" t="s">
+        <v>62</v>
+      </c>
+      <c r="I6" t="s">
+        <v>63</v>
+      </c>
+      <c r="J6" t="s">
         <v>64</v>
-      </c>
-      <c r="B6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" t="s">
-        <v>57</v>
-      </c>
-      <c r="D6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" t="s">
-        <v>65</v>
-      </c>
-      <c r="G6" t="s">
-        <v>60</v>
-      </c>
-      <c r="H6" t="s">
-        <v>66</v>
-      </c>
-      <c r="I6" t="s">
-        <v>67</v>
-      </c>
-      <c r="J6" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E7" t="s">
+        <v>6</v>
+      </c>
+      <c r="F7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H7" t="s">
+        <v>67</v>
+      </c>
+      <c r="I7" t="s">
+        <v>68</v>
+      </c>
+      <c r="J7" t="s">
         <v>69</v>
-      </c>
-      <c r="B7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" t="s">
-        <v>57</v>
-      </c>
-      <c r="D7" t="s">
-        <v>58</v>
-      </c>
-      <c r="E7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" t="s">
-        <v>70</v>
-      </c>
-      <c r="G7" t="s">
-        <v>60</v>
-      </c>
-      <c r="H7" t="s">
-        <v>71</v>
-      </c>
-      <c r="I7" t="s">
-        <v>72</v>
-      </c>
-      <c r="J7" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" t="s">
+        <v>71</v>
+      </c>
+      <c r="E8" t="s">
+        <v>6</v>
+      </c>
+      <c r="F8" t="s">
+        <v>72</v>
+      </c>
+      <c r="G8" t="s">
+        <v>56</v>
+      </c>
+      <c r="H8" t="s">
+        <v>73</v>
+      </c>
+      <c r="I8" t="s">
         <v>74</v>
       </c>
-      <c r="B8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" t="s">
-        <v>57</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="J8" t="s">
         <v>75</v>
-      </c>
-      <c r="E8" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" t="s">
-        <v>76</v>
-      </c>
-      <c r="G8" t="s">
-        <v>60</v>
-      </c>
-      <c r="H8" t="s">
-        <v>77</v>
-      </c>
-      <c r="I8" t="s">
-        <v>78</v>
-      </c>
-      <c r="J8" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C9" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" t="s">
+        <v>77</v>
+      </c>
+      <c r="G9" t="s">
+        <v>56</v>
+      </c>
+      <c r="H9" t="s">
+        <v>73</v>
+      </c>
+      <c r="I9" t="s">
+        <v>74</v>
+      </c>
+      <c r="J9" t="s">
         <v>75</v>
-      </c>
-      <c r="E9" t="s">
-        <v>10</v>
-      </c>
-      <c r="F9" t="s">
-        <v>81</v>
-      </c>
-      <c r="G9" t="s">
-        <v>60</v>
-      </c>
-      <c r="H9" t="s">
-        <v>77</v>
-      </c>
-      <c r="I9" t="s">
-        <v>78</v>
-      </c>
-      <c r="J9" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>79</v>
+      </c>
+      <c r="D10" t="s">
+        <v>80</v>
+      </c>
+      <c r="E10" t="s">
+        <v>6</v>
+      </c>
+      <c r="F10" t="s">
+        <v>81</v>
+      </c>
+      <c r="G10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H10" t="s">
         <v>82</v>
       </c>
-      <c r="B10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="I10" t="s">
         <v>83</v>
       </c>
-      <c r="D10" t="s">
+      <c r="J10" t="s">
         <v>84</v>
-      </c>
-      <c r="E10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F10" t="s">
-        <v>85</v>
-      </c>
-      <c r="G10" t="s">
-        <v>60</v>
-      </c>
-      <c r="H10" t="s">
-        <v>86</v>
-      </c>
-      <c r="I10" t="s">
-        <v>87</v>
-      </c>
-      <c r="J10" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>85</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" t="s">
+        <v>79</v>
+      </c>
+      <c r="D11" t="s">
+        <v>80</v>
+      </c>
+      <c r="E11" t="s">
+        <v>6</v>
+      </c>
+      <c r="F11" t="s">
+        <v>86</v>
+      </c>
+      <c r="G11" t="s">
+        <v>56</v>
+      </c>
+      <c r="H11" t="s">
+        <v>87</v>
+      </c>
+      <c r="I11" t="s">
+        <v>88</v>
+      </c>
+      <c r="J11" t="s">
         <v>89</v>
-      </c>
-      <c r="B11" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" t="s">
-        <v>83</v>
-      </c>
-      <c r="D11" t="s">
-        <v>84</v>
-      </c>
-      <c r="E11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11" t="s">
-        <v>90</v>
-      </c>
-      <c r="G11" t="s">
-        <v>60</v>
-      </c>
-      <c r="H11" t="s">
-        <v>91</v>
-      </c>
-      <c r="I11" t="s">
-        <v>92</v>
-      </c>
-      <c r="J11" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D12" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="E12" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F12" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="G12" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H12" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="I12" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="J12" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B13" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C13" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D13" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E13" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F13" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="G13" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H13" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="I13" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="J13" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C14" t="s">
+        <v>94</v>
+      </c>
+      <c r="D14" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" t="s">
         <v>98</v>
       </c>
-      <c r="D14" t="s">
-        <v>58</v>
-      </c>
-      <c r="E14" t="s">
-        <v>10</v>
-      </c>
-      <c r="F14" t="s">
-        <v>102</v>
-      </c>
       <c r="G14" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H14" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="I14" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="J14" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B15" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D15" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E15" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F15" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="G15" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H15" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="I15" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="J15" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D16" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E16" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F16" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="G16" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H16" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="I16" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="J16" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
+        <v>107</v>
+      </c>
+      <c r="B17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" t="s">
+        <v>54</v>
+      </c>
+      <c r="E17" t="s">
+        <v>6</v>
+      </c>
+      <c r="F17" t="s">
+        <v>108</v>
+      </c>
+      <c r="G17" t="s">
+        <v>109</v>
+      </c>
+      <c r="H17" t="s">
+        <v>110</v>
+      </c>
+      <c r="I17" t="s">
+        <v>74</v>
+      </c>
+      <c r="J17" t="s">
         <v>111</v>
-      </c>
-      <c r="B17" t="s">
-        <v>22</v>
-      </c>
-      <c r="C17" t="s">
-        <v>42</v>
-      </c>
-      <c r="D17" t="s">
-        <v>58</v>
-      </c>
-      <c r="E17" t="s">
-        <v>10</v>
-      </c>
-      <c r="F17" t="s">
-        <v>112</v>
-      </c>
-      <c r="G17" t="s">
-        <v>113</v>
-      </c>
-      <c r="H17" t="s">
-        <v>114</v>
-      </c>
-      <c r="I17" t="s">
-        <v>78</v>
-      </c>
-      <c r="J17" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C18" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D18" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E18" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F18" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G18" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H18" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="I18" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="J18" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B19" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C19" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D19" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E19" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F19" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="G19" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H19" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I19" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="J19" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B20" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C20" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D20" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E20" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F20" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="G20" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H20" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I20" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="J20" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -1912,50 +1912,50 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B2" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B3" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B4" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B5" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B6" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -1978,368 +1978,368 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C2" t="s">
+        <v>142</v>
+      </c>
+      <c r="D2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E2" t="s">
+        <v>144</v>
+      </c>
+      <c r="F2" t="s">
         <v>145</v>
-      </c>
-      <c r="C2" t="s">
-        <v>146</v>
-      </c>
-      <c r="D2" t="s">
-        <v>147</v>
-      </c>
-      <c r="E2" t="s">
-        <v>148</v>
-      </c>
-      <c r="F2" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B3" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="D3" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E3" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B4" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C4" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="D4" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E4" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B5" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C5" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D5" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E5" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B6" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C6" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D6" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E6" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="B7" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C7" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="D7" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E7" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="F7" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B8" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" t="s">
         <v>159</v>
       </c>
-      <c r="C8" t="s">
-        <v>163</v>
-      </c>
       <c r="D8" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E8" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B9" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C9" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="D9" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E9" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B10" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C10" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D10" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E10" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B11" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C11" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="D11" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E11" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B12" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C12" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="D12" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E12" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B13" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C13" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="D13" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E13" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B14" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C14" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D14" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E14" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B15" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C15" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D15" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E15" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B16" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C16" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D16" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E16" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B17" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C17" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D17" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E17" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B18" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C18" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D18" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E18" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B19" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C19" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D19" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E19" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B20" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C20" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="D20" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="E20" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B21" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C21" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D21" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="E21" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -2362,175 +2362,175 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B2" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="C2" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="D2" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="E2" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B3" t="s">
+        <v>187</v>
+      </c>
+      <c r="C3" t="s">
         <v>191</v>
       </c>
-      <c r="C3" t="s">
-        <v>195</v>
-      </c>
       <c r="D3" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="E3" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="B4" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="C4" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="D4" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="E4" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B5" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C5" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="D5" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="E5" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B6" t="s">
+        <v>195</v>
+      </c>
+      <c r="C6" t="s">
         <v>199</v>
       </c>
-      <c r="C6" t="s">
-        <v>203</v>
-      </c>
       <c r="D6" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="E6" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B7" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C7" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="D7" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="E7" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="B8" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C8" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="D8" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="E8" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="B9" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="C9" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="D9" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="E9" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="B10" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="C10" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="D10" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="E10" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -2553,153 +2553,153 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C2" t="s">
+        <v>211</v>
+      </c>
+      <c r="D2" t="s">
+        <v>212</v>
+      </c>
+      <c r="E2" t="s">
+        <v>144</v>
+      </c>
+      <c r="F2" t="s">
         <v>213</v>
-      </c>
-      <c r="B2" t="s">
-        <v>214</v>
-      </c>
-      <c r="C2" t="s">
-        <v>215</v>
-      </c>
-      <c r="D2" t="s">
-        <v>216</v>
-      </c>
-      <c r="E2" t="s">
-        <v>148</v>
-      </c>
-      <c r="F2" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="B3" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="C3" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="D3" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="E3" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="F3" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="B4" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="C4" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="D4" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="E4" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="F4" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="B5" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="C5" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="D5" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="E5" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="F5" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="B6" t="s">
+        <v>221</v>
+      </c>
+      <c r="C6" t="s">
         <v>225</v>
       </c>
-      <c r="C6" t="s">
-        <v>229</v>
-      </c>
       <c r="D6" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="E6" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="B7" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="C7" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="D7" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="E7" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="B8" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="C8" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="D8" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="E8" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: stabilize LLM evaluation framework v1
</commit_message>
<xml_diff>
--- a/datasets/Login_test_repository.xlsx
+++ b/datasets/Login_test_repository.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shivani Rampally\DeepEval-POC\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A857EEB-6045-4440-8AA5-A6BBB47C4BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{268309A9-4454-4FE9-8256-FC6839AD33E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_Requirements" sheetId="1" r:id="rId1"/>
-    <sheet name="02_GroundTruth_TestCases" sheetId="2" r:id="rId2"/>
-    <sheet name="03_GroundTruth_Metadata" sheetId="3" r:id="rId3"/>
+    <sheet name="02_Benchmark_TestCases" sheetId="2" r:id="rId2"/>
+    <sheet name="03_Benchmark_Metadata" sheetId="3" r:id="rId3"/>
     <sheet name="04_InputVariations" sheetId="4" r:id="rId4"/>
     <sheet name="05_UsabilityNavigation" sheetId="5" r:id="rId5"/>
     <sheet name="06_NonFunctional" sheetId="6" r:id="rId6"/>

</xml_diff>